<commit_message>
chore: update registrations data and excel spreadsheet
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -448,22 +448,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BR-2026-0001</v>
+        <v>BR-2026-0003</v>
       </c>
       <c r="C2" t="str">
-        <v>Sep 29, 2026, 10:41 AM (BST)</v>
+        <v>Sep 29, 2026, 11:22 AM (BST)</v>
       </c>
       <c r="D2" t="str">
-        <v>আহমেদ সাদিক</v>
+        <v>সাদিক আলম</v>
       </c>
       <c r="E2" t="str">
-        <v>01812345678</v>
+        <v>01717662350</v>
       </c>
       <c r="F2" t="str">
-        <v>sadiq@example.com</v>
+        <v>sadiq.alam@gmail.com</v>
       </c>
       <c r="G2" t="str">
-        <v>01812345678</v>
+        <v>01717662350</v>
       </c>
       <c r="H2" t="str">
         <v>Ticket Not Sent</v>
@@ -472,12 +472,76 @@
         <v>-</v>
       </c>
       <c r="J2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>BR-2026-0002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Sep 29, 2026, 11:00 AM (BST)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Sadiq test</v>
+      </c>
+      <c r="E3" t="str">
+        <v>01924572887</v>
+      </c>
+      <c r="F3" t="str">
+        <v>hello@sadiqalam.com</v>
+      </c>
+      <c r="G3" t="str">
+        <v>01711056474</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="I3" t="str">
+        <v>-</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BR-2026-0001</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sep 29, 2026, 10:41 AM (BST)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>আহমেদ সাদিক</v>
+      </c>
+      <c r="E4" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="F4" t="str">
+        <v>sadiq@example.com</v>
+      </c>
+      <c r="G4" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="I4" t="str">
+        <v>-</v>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear test data and initialize clean registration spreadsheet
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -443,105 +443,9 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>BR-2026-0003</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Sep 29, 2026, 11:22 AM (BST)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>সাদিক আলম</v>
-      </c>
-      <c r="E2" t="str">
-        <v>01717662350</v>
-      </c>
-      <c r="F2" t="str">
-        <v>sadiq.alam@gmail.com</v>
-      </c>
-      <c r="G2" t="str">
-        <v>01717662350</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Ticket Not Sent</v>
-      </c>
-      <c r="I2" t="str">
-        <v>-</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>BR-2026-0002</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Sep 29, 2026, 11:00 AM (BST)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Sadiq test</v>
-      </c>
-      <c r="E3" t="str">
-        <v>01924572887</v>
-      </c>
-      <c r="F3" t="str">
-        <v>hello@sadiqalam.com</v>
-      </c>
-      <c r="G3" t="str">
-        <v>01711056474</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Ticket Not Sent</v>
-      </c>
-      <c r="I3" t="str">
-        <v>-</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>BR-2026-0001</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sep 29, 2026, 10:41 AM (BST)</v>
-      </c>
-      <c r="D4" t="str">
-        <v>আহমেদ সাদিক</v>
-      </c>
-      <c r="E4" t="str">
-        <v>01812345678</v>
-      </c>
-      <c r="F4" t="str">
-        <v>sadiq@example.com</v>
-      </c>
-      <c r="G4" t="str">
-        <v>01812345678</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Ticket Not Sent</v>
-      </c>
-      <c r="I4" t="str">
-        <v>-</v>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add PDF ticket generator, DB cleanup scripts, and updated dependencies
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,18 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L6"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,27 +427,223 @@
         <v>Name (নাম)</v>
       </c>
       <c r="E1" t="str">
+        <v>Ticket Number</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Total Amount (মোট টাকা)</v>
+      </c>
+      <c r="G1" t="str">
         <v>WhatsApp Number (হোয়াটসঅ্যাপ)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Email (ইমেইল)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>bKash Number (বিকাশ নম্বর)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Status</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Ticket Code</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>BR-2026-0009</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Emon Rahman</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>500</v>
+      </c>
+      <c r="G2" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="H2" t="str">
+        <v>biswas.lipika05@gmail.com</v>
+      </c>
+      <c r="I2" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K2" t="str">
+        <v>-</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>BR-2026-0008</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ferdowsi Rita</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>500</v>
+      </c>
+      <c r="G3" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="H3" t="str">
+        <v>ferdowsi.rita@gmail.com</v>
+      </c>
+      <c r="I3" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K3" t="str">
+        <v>-</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BR-2026-0007</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>মল্লিকা</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="H4" t="str">
+        <v>mallikarikta142@gmail.com</v>
+      </c>
+      <c r="I4" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K4" t="str">
+        <v>-</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>BR-2026-0004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Anindita Bhattacharjee</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>500</v>
+      </c>
+      <c r="G5" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="H5" t="str">
+        <v>anindita1603@gmail.com</v>
+      </c>
+      <c r="I5" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K5" t="str">
+        <v>-</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BR-2026-0002</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sep 30, 2026, 02:12 AM (BST)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>সাবিনা ইয়াসমিন</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>500</v>
+      </c>
+      <c r="G6" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="H6" t="str">
+        <v>sabinakakoli@gmail.com</v>
+      </c>
+      <c r="I6" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K6" t="str">
+        <v>-</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update email templates and add ticket scripts
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -579,10 +579,10 @@
         <v>Anindita Bhattacharjee</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G5" t="str">
         <v>01711107102</v>

</xml_diff>

<commit_message>
Mark participants with sent tickets as Mail Sent, update database and admin panel
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L23"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -456,13 +456,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BR-2026-0009</v>
+        <v>BR-2026-0022</v>
       </c>
       <c r="C2" t="str">
-        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+        <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D2" t="str">
-        <v>Emon Rahman</v>
+        <v>Mahenaw Wara</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -471,22 +471,22 @@
         <v>500</v>
       </c>
       <c r="G2" t="str">
-        <v>01971010112</v>
+        <v>01030300120</v>
       </c>
       <c r="H2" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>manana.manamaya@gmail.com</v>
       </c>
       <c r="I2" t="str">
-        <v>01971010112</v>
+        <v>01030300120</v>
       </c>
       <c r="J2" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K2" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-02</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="3">
@@ -494,13 +494,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>BR-2026-0008</v>
+        <v>BR-2026-0021</v>
       </c>
       <c r="C3" t="str">
-        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+        <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D3" t="str">
-        <v>Ferdowsi Rita</v>
+        <v>Ferdoushi Begum</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -509,22 +509,22 @@
         <v>500</v>
       </c>
       <c r="G3" t="str">
-        <v>01732770345</v>
+        <v>01717144778</v>
       </c>
       <c r="H3" t="str">
-        <v>ferdowsi.rita@gmail.com</v>
+        <v>ferdoushi@yahoo.com</v>
       </c>
       <c r="I3" t="str">
-        <v>01732770345</v>
+        <v>01717144778</v>
       </c>
       <c r="J3" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K3" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-01</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="4">
@@ -532,28 +532,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>BR-2026-0007</v>
+        <v>BR-2026-0020</v>
       </c>
       <c r="C4" t="str">
-        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+        <v>Oct 04, 2026, 11:43 AM (BST)</v>
       </c>
       <c r="D4" t="str">
-        <v>মল্লিকা</v>
+        <v>Delwar Hossain</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G4" t="str">
-        <v>01716550859</v>
+        <v>01715458432</v>
       </c>
       <c r="H4" t="str">
-        <v>mallikarikta142@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I4" t="str">
-        <v>01716550859</v>
+        <v>01715458432</v>
       </c>
       <c r="J4" t="str">
         <v>Ticket Not Sent</v>
@@ -570,31 +570,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>BR-2026-0004</v>
+        <v>BR-2026-0019</v>
       </c>
       <c r="C5" t="str">
-        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+        <v>Oct 04, 2026, 10:35 AM (BST)</v>
       </c>
       <c r="D5" t="str">
-        <v>Anindita Bhattacharjee</v>
+        <v>ইলোরা</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G5" t="str">
-        <v>01711107102</v>
+        <v>01730599329</v>
       </c>
       <c r="H5" t="str">
-        <v>anindita1603@gmail.com</v>
+        <v>sselora.harmony19@gmail.com</v>
       </c>
       <c r="I5" t="str">
-        <v>01711107102</v>
+        <v>01730599329</v>
       </c>
       <c r="J5" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K5" t="str">
         <v>-</v>
@@ -608,42 +608,688 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
+        <v>BR-2026-0018</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Oct 03, 2026, 08:34 PM (BST)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kanika Chakraborty</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>2000</v>
+      </c>
+      <c r="G6" t="str">
+        <v>01713379897</v>
+      </c>
+      <c r="H6" t="str">
+        <v>borty.kanika@yahoo.com</v>
+      </c>
+      <c r="I6" t="str">
+        <v>01713379897</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K6" t="str">
+        <v>-</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BR-2026-0017</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Oct 03, 2026, 07:54 PM (BST)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Sayema Mukarrama</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>500</v>
+      </c>
+      <c r="G7" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="H7" t="str">
+        <v>sayema14bd@gmail.com</v>
+      </c>
+      <c r="I7" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K7" t="str">
+        <v>-</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BR-2026-0016</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Oct 03, 2026, 07:41 PM (BST)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Sayema Mukarrama</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>500</v>
+      </c>
+      <c r="G8" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="H8" t="str">
+        <v>sayema14bd@gmail.com</v>
+      </c>
+      <c r="I8" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K8" t="str">
+        <v>-</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BR-2026-0015</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Oct 03, 2026, 07:13 PM (BST)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>কাজী নজরুল ইসলাম</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>500</v>
+      </c>
+      <c r="G9" t="str">
+        <v>01845972555</v>
+      </c>
+      <c r="H9" t="str">
+        <v>sarothy@gmail.com</v>
+      </c>
+      <c r="I9" t="str">
+        <v>01845972555</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K9" t="str">
+        <v>-</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BR-2026-0014</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Oct 03, 2026, 01:27 PM (BST)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>444</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>500</v>
+      </c>
+      <c r="G10" t="str">
+        <v>01712345678</v>
+      </c>
+      <c r="H10" t="str">
+        <v>kentkouh+otybu@gmail.com</v>
+      </c>
+      <c r="I10" t="str">
+        <v>01712345678</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K10" t="str">
+        <v>-</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>BR-2026-0013</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Oct 03, 2026, 12:06 PM (BST)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Ferdowsi Rita</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>1000</v>
+      </c>
+      <c r="G11" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="H11" t="str">
+        <v>ferdowsi.rita@gmail.com</v>
+      </c>
+      <c r="I11" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K11" t="str">
+        <v>-</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>BR-2026-0012</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Oct 02, 2026, 11:09 PM (BST)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>মো: হাবিবুর রহমান শিনু</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>500</v>
+      </c>
+      <c r="G12" t="str">
+        <v>01712286494</v>
+      </c>
+      <c r="H12" t="str">
+        <v>sassybd1978@gmail.com</v>
+      </c>
+      <c r="I12" t="str">
+        <v>01712286494</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K12" t="str">
+        <v>-</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>BR-2026-0011</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Oct 02, 2026, 08:09 PM (BST)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Anowar Hossain</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>1000</v>
+      </c>
+      <c r="G13" t="str">
+        <v>01711080069</v>
+      </c>
+      <c r="H13" t="str">
+        <v>anowarstories@gmail.com</v>
+      </c>
+      <c r="I13" t="str">
+        <v>01711080069</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K13" t="str">
+        <v>-</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BR-2026-0010</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Oct 02, 2026, 06:31 PM (BST)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Shawli Jharna</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>500</v>
+      </c>
+      <c r="G14" t="str">
+        <v>01313357635</v>
+      </c>
+      <c r="H14" t="str">
+        <v>shawli.jharna@yahoo.com</v>
+      </c>
+      <c r="I14" t="str">
+        <v>01313357635</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K14" t="str">
+        <v>-</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>BR-2026-0009</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Oct 02, 2026, 04:52 PM (BST)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>ফারজানা মাসুদ</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>500</v>
+      </c>
+      <c r="G15" t="str">
+        <v>01822055931</v>
+      </c>
+      <c r="H15" t="str">
+        <v>farjana.masud@plpg.com.bd</v>
+      </c>
+      <c r="I15" t="str">
+        <v>01822055931</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K15" t="str">
+        <v>-</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>BR-2026-0008</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Oct 02, 2026, 12:51 AM (BST)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Farhana Hafiz Tania</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>500</v>
+      </c>
+      <c r="G16" t="str">
+        <v>01713060155</v>
+      </c>
+      <c r="H16" t="str">
+        <v>fhafiz2006@gmail.com</v>
+      </c>
+      <c r="I16" t="str">
+        <v>01713046659</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K16" t="str">
+        <v>-</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>BR-2026-0007</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Oct 01, 2026, 11:38 PM (BST)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Nahida Parvin</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>500</v>
+      </c>
+      <c r="G17" t="str">
+        <v>01764198696</v>
+      </c>
+      <c r="H17" t="str">
+        <v>avra.bhattacharjee@gmail.com</v>
+      </c>
+      <c r="I17" t="str">
+        <v>01713244349</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K17" t="str">
+        <v>-</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>BR-2026-0006</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Oct 01, 2026, 05:59 PM (BST)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Moni Akter and Shela</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>1000</v>
+      </c>
+      <c r="G18" t="str">
+        <v>01718277527</v>
+      </c>
+      <c r="H18" t="str">
+        <v>biswas.lipika05@gmail.com</v>
+      </c>
+      <c r="I18" t="str">
+        <v>01715458432</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K18" t="str">
+        <v>-</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>BR-2026-0009</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Emon Rahman</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>500</v>
+      </c>
+      <c r="G19" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="H19" t="str">
+        <v>biswas.lipika05@gmail.com</v>
+      </c>
+      <c r="I19" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K19" t="str">
+        <v>-</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>BR-2026-0008</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Ferdowsi Rita</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>500</v>
+      </c>
+      <c r="G20" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="H20" t="str">
+        <v>ferdowsi.rita@gmail.com</v>
+      </c>
+      <c r="I20" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K20" t="str">
+        <v>-</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>BR-2026-0007</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>মল্লিকা</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>1000</v>
+      </c>
+      <c r="G21" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="H21" t="str">
+        <v>mallikarikta142@gmail.com</v>
+      </c>
+      <c r="I21" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K21" t="str">
+        <v>-</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>BR-2026-0004</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Anindita Bhattacharjee</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>1000</v>
+      </c>
+      <c r="G22" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="H22" t="str">
+        <v>anindita1603@gmail.com</v>
+      </c>
+      <c r="I22" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K22" t="str">
+        <v>-</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
         <v>BR-2026-0002</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C23" t="str">
         <v>Sep 30, 2026, 02:12 AM (BST)</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D23" t="str">
         <v>সাবিনা ইয়াসমিন</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>500</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>500</v>
+      </c>
+      <c r="G23" t="str">
         <v>01812345678</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H23" t="str">
         <v>sabinakakoli@gmail.com</v>
       </c>
-      <c r="I6" t="str">
+      <c r="I23" t="str">
         <v>01812345678</v>
       </c>
-      <c r="J6" t="str">
-        <v>Ticket Not Sent</v>
-      </c>
-      <c r="K6" t="str">
-        <v>-</v>
-      </c>
-      <c r="L6" t="str">
+      <c r="J23" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K23" t="str">
+        <v>-</v>
+      </c>
+      <c r="L23" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Close online registration, disable ticket inputs with notice, and generate 8oct2026 tickets
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L39"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -456,13 +456,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BR-2026-0022</v>
+        <v>BR-2026-0038</v>
       </c>
       <c r="C2" t="str">
-        <v>Oct 04, 2026, 05:13 PM (BST)</v>
+        <v>Oct 08, 2026, 08:27 PM (BST)</v>
       </c>
       <c r="D2" t="str">
-        <v>Mahenaw Wara</v>
+        <v>Tahera Jabeen</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -471,22 +471,22 @@
         <v>500</v>
       </c>
       <c r="G2" t="str">
-        <v>01030300120</v>
+        <v>01715325576</v>
       </c>
       <c r="H2" t="str">
-        <v>manana.manamaya@gmail.com</v>
+        <v>taherajabeen@yahoo.com</v>
       </c>
       <c r="I2" t="str">
-        <v>01030300120</v>
+        <v>01715325576</v>
       </c>
       <c r="J2" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K2" t="str">
-        <v>BR-OFFLINE-02</v>
+        <v>-</v>
       </c>
       <c r="L2" t="str">
-        <v>Offline CSV registration</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -494,37 +494,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>BR-2026-0021</v>
+        <v>BR-2026-0037</v>
       </c>
       <c r="C3" t="str">
-        <v>Oct 04, 2026, 05:13 PM (BST)</v>
+        <v>Oct 08, 2026, 07:42 PM (BST)</v>
       </c>
       <c r="D3" t="str">
-        <v>Ferdoushi Begum</v>
+        <v>Biplob Kumar Hazra</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="str">
-        <v>01717144778</v>
+        <v>01733454575</v>
       </c>
       <c r="H3" t="str">
-        <v>ferdoushi@yahoo.com</v>
+        <v>hazrabiplob@yahoo.com</v>
       </c>
       <c r="I3" t="str">
-        <v>01717144778</v>
+        <v>01733454575</v>
       </c>
       <c r="J3" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K3" t="str">
-        <v>BR-OFFLINE-01</v>
+        <v>-</v>
       </c>
       <c r="L3" t="str">
-        <v>Offline CSV registration</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>BR-2026-0020</v>
+        <v>BR-2026-0036</v>
       </c>
       <c r="C4" t="str">
-        <v>Oct 04, 2026, 11:43 AM (BST)</v>
+        <v>Oct 08, 2026, 05:04 PM (BST)</v>
       </c>
       <c r="D4" t="str">
-        <v>Delwar Hossain</v>
+        <v>মাহবুবা রাখি</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -547,13 +547,13 @@
         <v>500</v>
       </c>
       <c r="G4" t="str">
-        <v>01715458432</v>
+        <v>01615253954</v>
       </c>
       <c r="H4" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>mahbubaalam300@gmail.com</v>
       </c>
       <c r="I4" t="str">
-        <v>01715458432</v>
+        <v>01615253954</v>
       </c>
       <c r="J4" t="str">
         <v>Ticket Not Sent</v>
@@ -570,13 +570,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>BR-2026-0019</v>
+        <v>BR-2026-0035</v>
       </c>
       <c r="C5" t="str">
-        <v>Oct 04, 2026, 10:35 AM (BST)</v>
+        <v>Oct 08, 2026, 05:04 PM (BST)</v>
       </c>
       <c r="D5" t="str">
-        <v>ইলোরা</v>
+        <v>মাহবুবা রাখি</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -585,16 +585,16 @@
         <v>500</v>
       </c>
       <c r="G5" t="str">
-        <v>01730599329</v>
+        <v>01615253954</v>
       </c>
       <c r="H5" t="str">
-        <v>sselora.harmony19@gmail.com</v>
+        <v>mahbubaalam300@gmail.com</v>
       </c>
       <c r="I5" t="str">
-        <v>01730599329</v>
+        <v>01615253954</v>
       </c>
       <c r="J5" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K5" t="str">
         <v>-</v>
@@ -608,31 +608,31 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>BR-2026-0018</v>
+        <v>BR-2026-0034</v>
       </c>
       <c r="C6" t="str">
-        <v>Oct 03, 2026, 08:34 PM (BST)</v>
+        <v>Oct 08, 2026, 05:03 PM (BST)</v>
       </c>
       <c r="D6" t="str">
-        <v>Kanika Chakraborty</v>
+        <v>মাহবুবা রাখি</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G6" t="str">
-        <v>01713379897</v>
+        <v>01615253954</v>
       </c>
       <c r="H6" t="str">
-        <v>borty.kanika@yahoo.com</v>
+        <v>mahbubaalam300@gmail.com</v>
       </c>
       <c r="I6" t="str">
-        <v>01713379897</v>
+        <v>01615253954</v>
       </c>
       <c r="J6" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K6" t="str">
         <v>-</v>
@@ -646,13 +646,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>BR-2026-0017</v>
+        <v>BR-2026-0033</v>
       </c>
       <c r="C7" t="str">
-        <v>Oct 03, 2026, 07:54 PM (BST)</v>
+        <v>Oct 08, 2026, 04:06 PM (BST)</v>
       </c>
       <c r="D7" t="str">
-        <v>Sayema Mukarrama</v>
+        <v>Suraiya Mozammel</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -661,16 +661,16 @@
         <v>500</v>
       </c>
       <c r="G7" t="str">
-        <v>01973091880</v>
+        <v>01712963636</v>
       </c>
       <c r="H7" t="str">
-        <v>sayema14bd@gmail.com</v>
+        <v>srabani.s@brac.net</v>
       </c>
       <c r="I7" t="str">
-        <v>01973091880</v>
+        <v>01717662350</v>
       </c>
       <c r="J7" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K7" t="str">
         <v>-</v>
@@ -684,13 +684,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>BR-2026-0016</v>
+        <v>BR-2026-0032</v>
       </c>
       <c r="C8" t="str">
-        <v>Oct 03, 2026, 07:41 PM (BST)</v>
+        <v>Oct 08, 2026, 02:19 PM (BST)</v>
       </c>
       <c r="D8" t="str">
-        <v>Sayema Mukarrama</v>
+        <v>Mohammed Shoeb</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -699,13 +699,13 @@
         <v>500</v>
       </c>
       <c r="G8" t="str">
-        <v>01973091880</v>
+        <v>01615253954</v>
       </c>
       <c r="H8" t="str">
-        <v>sayema14bd@gmail.com</v>
+        <v>shoeb@trtradingbd.com</v>
       </c>
       <c r="I8" t="str">
-        <v>01973091880</v>
+        <v>01615253954</v>
       </c>
       <c r="J8" t="str">
         <v>Ticket Not Sent</v>
@@ -722,31 +722,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>BR-2026-0015</v>
+        <v>BR-2026-0031</v>
       </c>
       <c r="C9" t="str">
-        <v>Oct 03, 2026, 07:13 PM (BST)</v>
+        <v>Oct 08, 2026, 11:42 AM (BST)</v>
       </c>
       <c r="D9" t="str">
-        <v>কাজী নজরুল ইসলাম</v>
+        <v>Kishower Amin</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G9" t="str">
-        <v>01845972555</v>
+        <v>01766903903</v>
       </c>
       <c r="H9" t="str">
-        <v>sarothy@gmail.com</v>
+        <v>kishowerca@gmail.com</v>
       </c>
       <c r="I9" t="str">
-        <v>01845972555</v>
+        <v>01766903903</v>
       </c>
       <c r="J9" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K9" t="str">
         <v>-</v>
@@ -760,13 +760,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>BR-2026-0014</v>
+        <v>BR-2026-0030</v>
       </c>
       <c r="C10" t="str">
-        <v>Oct 03, 2026, 01:27 PM (BST)</v>
+        <v>Oct 07, 2026, 10:51 PM (BST)</v>
       </c>
       <c r="D10" t="str">
-        <v>444</v>
+        <v>Juthi</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -775,13 +775,13 @@
         <v>500</v>
       </c>
       <c r="G10" t="str">
-        <v>01712345678</v>
+        <v>01715458432</v>
       </c>
       <c r="H10" t="str">
-        <v>kentkouh+otybu@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I10" t="str">
-        <v>01712345678</v>
+        <v>01715458432</v>
       </c>
       <c r="J10" t="str">
         <v>Ticket Not Sent</v>
@@ -798,31 +798,31 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>BR-2026-0013</v>
+        <v>BR-2026-0029</v>
       </c>
       <c r="C11" t="str">
-        <v>Oct 03, 2026, 12:06 PM (BST)</v>
+        <v>Oct 07, 2026, 03:17 PM (BST)</v>
       </c>
       <c r="D11" t="str">
-        <v>Ferdowsi Rita</v>
+        <v>Bidhan Chandra Pal</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G11" t="str">
-        <v>01732770345</v>
+        <v>01730715222</v>
       </c>
       <c r="H11" t="str">
-        <v>ferdowsi.rita@gmail.com</v>
+        <v>bidhan.probhaaurora@gmail.com</v>
       </c>
       <c r="I11" t="str">
-        <v>01732770345</v>
+        <v>01730715222</v>
       </c>
       <c r="J11" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K11" t="str">
         <v>-</v>
@@ -836,37 +836,37 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>BR-2026-0012</v>
+        <v>BR-OFFLINE-04</v>
       </c>
       <c r="C12" t="str">
-        <v>Oct 02, 2026, 11:09 PM (BST)</v>
+        <v>Oct 07, 2026, 12:01 AM (BST)</v>
       </c>
       <c r="D12" t="str">
-        <v>মো: হাবিবুর রহমান শিনু</v>
+        <v>Shahajadi Begum</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F12">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G12" t="str">
-        <v>01712286494</v>
+        <v/>
       </c>
       <c r="H12" t="str">
-        <v>sassybd1978@gmail.com</v>
+        <v>shahajadibegum@gmail.com</v>
       </c>
       <c r="I12" t="str">
-        <v>01712286494</v>
+        <v/>
       </c>
       <c r="J12" t="str">
         <v>Mail Sent</v>
       </c>
       <c r="K12" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-04</v>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="13">
@@ -874,37 +874,37 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>BR-2026-0011</v>
+        <v>BR-OFFLINE-03</v>
       </c>
       <c r="C13" t="str">
-        <v>Oct 02, 2026, 08:09 PM (BST)</v>
+        <v>Oct 07, 2026, 12:01 AM (BST)</v>
       </c>
       <c r="D13" t="str">
-        <v>Anowar Hossain</v>
+        <v>Abid Aziz</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G13" t="str">
-        <v>01711080069</v>
+        <v/>
       </c>
       <c r="H13" t="str">
-        <v>anowarstories@gmail.com</v>
+        <v>aby9029@gmail.com</v>
       </c>
       <c r="I13" t="str">
-        <v>01711080069</v>
+        <v/>
       </c>
       <c r="J13" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K13" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-03</v>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="14">
@@ -912,28 +912,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>BR-2026-0010</v>
+        <v>BR-2026-0026</v>
       </c>
       <c r="C14" t="str">
-        <v>Oct 02, 2026, 06:31 PM (BST)</v>
+        <v>Oct 06, 2026, 11:24 PM (BST)</v>
       </c>
       <c r="D14" t="str">
-        <v>Shawli Jharna</v>
+        <v>Saud Bin Jahan (Susan)</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G14" t="str">
-        <v>01313357635</v>
+        <v>01714100924</v>
       </c>
       <c r="H14" t="str">
-        <v>shawli.jharna@yahoo.com</v>
+        <v>saud.jahan@outlook.com</v>
       </c>
       <c r="I14" t="str">
-        <v>01313357635</v>
+        <v>01714100924</v>
       </c>
       <c r="J14" t="str">
         <v>Ticket Not Sent</v>
@@ -950,13 +950,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>BR-2026-0009</v>
+        <v>BR-2026-0025</v>
       </c>
       <c r="C15" t="str">
-        <v>Oct 02, 2026, 04:52 PM (BST)</v>
+        <v>Oct 06, 2026, 11:03 PM (BST)</v>
       </c>
       <c r="D15" t="str">
-        <v>ফারজানা মাসুদ</v>
+        <v>Joya Tasnim</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -965,13 +965,13 @@
         <v>500</v>
       </c>
       <c r="G15" t="str">
-        <v>01822055931</v>
+        <v>01911586356</v>
       </c>
       <c r="H15" t="str">
-        <v>farjana.masud@plpg.com.bd</v>
+        <v>joyatasnim229@gmail.com</v>
       </c>
       <c r="I15" t="str">
-        <v>01822055931</v>
+        <v>01876892247</v>
       </c>
       <c r="J15" t="str">
         <v>Ticket Not Sent</v>
@@ -988,28 +988,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>BR-2026-0008</v>
+        <v>BR-2026-0024</v>
       </c>
       <c r="C16" t="str">
-        <v>Oct 02, 2026, 12:51 AM (BST)</v>
+        <v>Oct 06, 2026, 10:23 AM (BST)</v>
       </c>
       <c r="D16" t="str">
-        <v>Farhana Hafiz Tania</v>
+        <v>Saikat Shubhra Aich</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G16" t="str">
-        <v>01713060155</v>
+        <v>01712032080</v>
       </c>
       <c r="H16" t="str">
-        <v>fhafiz2006@gmail.com</v>
+        <v>ssam99@gmail.com</v>
       </c>
       <c r="I16" t="str">
-        <v>01713046659</v>
+        <v>01712032080</v>
       </c>
       <c r="J16" t="str">
         <v>Ticket Not Sent</v>
@@ -1026,31 +1026,31 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>BR-2026-0007</v>
+        <v>BR-2026-0023</v>
       </c>
       <c r="C17" t="str">
-        <v>Oct 01, 2026, 11:38 PM (BST)</v>
+        <v>Oct 05, 2026, 09:13 AM (BST)</v>
       </c>
       <c r="D17" t="str">
-        <v>Nahida Parvin</v>
+        <v>Shariful Islam</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G17" t="str">
-        <v>01764198696</v>
+        <v>01778580756</v>
       </c>
       <c r="H17" t="str">
-        <v>avra.bhattacharjee@gmail.com</v>
+        <v>sharif1658@gmail.com</v>
       </c>
       <c r="I17" t="str">
-        <v>01713244349</v>
+        <v>01778580756</v>
       </c>
       <c r="J17" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K17" t="str">
         <v>-</v>
@@ -1064,37 +1064,37 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>BR-2026-0006</v>
+        <v>BR-2026-0022</v>
       </c>
       <c r="C18" t="str">
-        <v>Oct 01, 2026, 05:59 PM (BST)</v>
+        <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D18" t="str">
-        <v>Moni Akter and Shela</v>
+        <v>Mahenaw Wara</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G18" t="str">
-        <v>01718277527</v>
+        <v>01030300120</v>
       </c>
       <c r="H18" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>manana.manamaya@gmail.com</v>
       </c>
       <c r="I18" t="str">
-        <v>01715458432</v>
+        <v>01030300120</v>
       </c>
       <c r="J18" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K18" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-02</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="19">
@@ -1102,13 +1102,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>BR-2026-0009</v>
+        <v>BR-2026-0021</v>
       </c>
       <c r="C19" t="str">
-        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+        <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D19" t="str">
-        <v>Emon Rahman</v>
+        <v>Ferdoushi Begum</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1117,22 +1117,22 @@
         <v>500</v>
       </c>
       <c r="G19" t="str">
-        <v>01971010112</v>
+        <v>01717144778</v>
       </c>
       <c r="H19" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>ferdoushi@yahoo.com</v>
       </c>
       <c r="I19" t="str">
-        <v>01971010112</v>
+        <v>01717144778</v>
       </c>
       <c r="J19" t="str">
         <v>Mail Sent</v>
       </c>
       <c r="K19" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-01</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="20">
@@ -1140,13 +1140,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>BR-2026-0008</v>
+        <v>BR-2026-0020</v>
       </c>
       <c r="C20" t="str">
-        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+        <v>Oct 04, 2026, 11:43 AM (BST)</v>
       </c>
       <c r="D20" t="str">
-        <v>Ferdowsi Rita</v>
+        <v>Delwar Hossain</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1155,13 +1155,13 @@
         <v>500</v>
       </c>
       <c r="G20" t="str">
-        <v>01732770345</v>
+        <v>01715458432</v>
       </c>
       <c r="H20" t="str">
-        <v>ferdowsi.rita@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I20" t="str">
-        <v>01732770345</v>
+        <v>01715458432</v>
       </c>
       <c r="J20" t="str">
         <v>Ticket Not Sent</v>
@@ -1178,31 +1178,31 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>BR-2026-0007</v>
+        <v>BR-2026-0019</v>
       </c>
       <c r="C21" t="str">
-        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+        <v>Oct 04, 2026, 10:35 AM (BST)</v>
       </c>
       <c r="D21" t="str">
-        <v>মল্লিকা</v>
+        <v>ইলোরা</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G21" t="str">
-        <v>01716550859</v>
+        <v>01730599329</v>
       </c>
       <c r="H21" t="str">
-        <v>mallikarikta142@gmail.com</v>
+        <v>sselora.harmony19@gmail.com</v>
       </c>
       <c r="I21" t="str">
-        <v>01716550859</v>
+        <v>01730599329</v>
       </c>
       <c r="J21" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K21" t="str">
         <v>-</v>
@@ -1216,28 +1216,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>BR-2026-0004</v>
+        <v>BR-2026-0018</v>
       </c>
       <c r="C22" t="str">
-        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+        <v>Oct 03, 2026, 08:34 PM (BST)</v>
       </c>
       <c r="D22" t="str">
-        <v>Anindita Bhattacharjee</v>
+        <v>Kanika Chakraborty</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F22">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G22" t="str">
-        <v>01711107102</v>
+        <v>01713379897</v>
       </c>
       <c r="H22" t="str">
-        <v>anindita1603@gmail.com</v>
+        <v>borty.kanika@yahoo.com</v>
       </c>
       <c r="I22" t="str">
-        <v>01711107102</v>
+        <v>01713379897</v>
       </c>
       <c r="J22" t="str">
         <v>Mail Sent</v>
@@ -1254,13 +1254,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>BR-2026-0002</v>
+        <v>BR-2026-0017</v>
       </c>
       <c r="C23" t="str">
-        <v>Sep 30, 2026, 02:12 AM (BST)</v>
+        <v>Oct 03, 2026, 07:54 PM (BST)</v>
       </c>
       <c r="D23" t="str">
-        <v>সাবিনা ইয়াসমিন</v>
+        <v>Sayema Mukarrama</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1269,13 +1269,13 @@
         <v>500</v>
       </c>
       <c r="G23" t="str">
-        <v>01812345678</v>
+        <v>01973091880</v>
       </c>
       <c r="H23" t="str">
-        <v>sabinakakoli@gmail.com</v>
+        <v>sayema14bd@gmail.com</v>
       </c>
       <c r="I23" t="str">
-        <v>01812345678</v>
+        <v>01973091880</v>
       </c>
       <c r="J23" t="str">
         <v>Mail Sent</v>
@@ -1287,9 +1287,617 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>BR-2026-0016</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Oct 03, 2026, 07:41 PM (BST)</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Sayema Mukarrama</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>500</v>
+      </c>
+      <c r="G24" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="H24" t="str">
+        <v>sayema14bd@gmail.com</v>
+      </c>
+      <c r="I24" t="str">
+        <v>01973091880</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K24" t="str">
+        <v>-</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>BR-2026-0015</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Oct 03, 2026, 07:13 PM (BST)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>কাজী নজরুল ইসলাম</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>500</v>
+      </c>
+      <c r="G25" t="str">
+        <v>01845972555</v>
+      </c>
+      <c r="H25" t="str">
+        <v>sarothy@gmail.com</v>
+      </c>
+      <c r="I25" t="str">
+        <v>01845972555</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K25" t="str">
+        <v>-</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>BR-2026-0014</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Oct 03, 2026, 01:27 PM (BST)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>444</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>500</v>
+      </c>
+      <c r="G26" t="str">
+        <v>01712345678</v>
+      </c>
+      <c r="H26" t="str">
+        <v>kentkouh+otybu@gmail.com</v>
+      </c>
+      <c r="I26" t="str">
+        <v>01712345678</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K26" t="str">
+        <v>-</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>BR-2026-0013</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Oct 03, 2026, 12:06 PM (BST)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Ferdowsi Rita</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+      <c r="F27">
+        <v>1000</v>
+      </c>
+      <c r="G27" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="H27" t="str">
+        <v>ferdowsi.rita@gmail.com</v>
+      </c>
+      <c r="I27" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K27" t="str">
+        <v>-</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>BR-2026-0012</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Oct 02, 2026, 11:09 PM (BST)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>মো: হাবিবুর রহমান শিনু</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>500</v>
+      </c>
+      <c r="G28" t="str">
+        <v>01712286494</v>
+      </c>
+      <c r="H28" t="str">
+        <v>sassybd1978@gmail.com</v>
+      </c>
+      <c r="I28" t="str">
+        <v>01712286494</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K28" t="str">
+        <v>-</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>BR-2026-0011</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Oct 02, 2026, 08:09 PM (BST)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Anowar Hossain</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29">
+        <v>1000</v>
+      </c>
+      <c r="G29" t="str">
+        <v>01711080069</v>
+      </c>
+      <c r="H29" t="str">
+        <v>anowarstories@gmail.com</v>
+      </c>
+      <c r="I29" t="str">
+        <v>01711080069</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K29" t="str">
+        <v>-</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>BR-2026-0010</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Oct 02, 2026, 06:31 PM (BST)</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Shawli Jharna</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>500</v>
+      </c>
+      <c r="G30" t="str">
+        <v>01313357635</v>
+      </c>
+      <c r="H30" t="str">
+        <v>shawli.jharna@yahoo.com</v>
+      </c>
+      <c r="I30" t="str">
+        <v>01313357635</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K30" t="str">
+        <v>-</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>BR-2026-0009</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Oct 02, 2026, 04:52 PM (BST)</v>
+      </c>
+      <c r="D31" t="str">
+        <v>ফারজানা মাসুদ</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>500</v>
+      </c>
+      <c r="G31" t="str">
+        <v>01822055931</v>
+      </c>
+      <c r="H31" t="str">
+        <v>farjana.masud@plpg.com.bd</v>
+      </c>
+      <c r="I31" t="str">
+        <v>01822055931</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K31" t="str">
+        <v>-</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>BR-2026-0008</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Oct 02, 2026, 12:51 AM (BST)</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Farhana Hafiz Tania</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>500</v>
+      </c>
+      <c r="G32" t="str">
+        <v>01713060155</v>
+      </c>
+      <c r="H32" t="str">
+        <v>fhafiz2006@gmail.com</v>
+      </c>
+      <c r="I32" t="str">
+        <v>01713046659</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K32" t="str">
+        <v>-</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>BR-2026-0007</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Oct 01, 2026, 11:38 PM (BST)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Nahida Parvin</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>500</v>
+      </c>
+      <c r="G33" t="str">
+        <v>01764198696</v>
+      </c>
+      <c r="H33" t="str">
+        <v>avra.bhattacharjee@gmail.com</v>
+      </c>
+      <c r="I33" t="str">
+        <v>01713244349</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K33" t="str">
+        <v>-</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>BR-2026-0006</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Oct 01, 2026, 05:59 PM (BST)</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Moni Akter and Shela</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+      <c r="F34">
+        <v>1000</v>
+      </c>
+      <c r="G34" t="str">
+        <v>01718277527</v>
+      </c>
+      <c r="H34" t="str">
+        <v>biswas.lipika05@gmail.com</v>
+      </c>
+      <c r="I34" t="str">
+        <v>01715458432</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K34" t="str">
+        <v>-</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>BR-2026-0009</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Emon Rahman</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>500</v>
+      </c>
+      <c r="G35" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="H35" t="str">
+        <v>biswas.lipika05@gmail.com</v>
+      </c>
+      <c r="I35" t="str">
+        <v>01971010112</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K35" t="str">
+        <v>-</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>BR-2026-0008</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Ferdowsi Rita</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
+        <v>500</v>
+      </c>
+      <c r="G36" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="H36" t="str">
+        <v>ferdowsi.rita@gmail.com</v>
+      </c>
+      <c r="I36" t="str">
+        <v>01732770345</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K36" t="str">
+        <v>-</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>BR-2026-0007</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+      </c>
+      <c r="D37" t="str">
+        <v>মল্লিকা</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>1000</v>
+      </c>
+      <c r="G37" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="H37" t="str">
+        <v>mallikarikta142@gmail.com</v>
+      </c>
+      <c r="I37" t="str">
+        <v>01716550859</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Ticket Not Sent</v>
+      </c>
+      <c r="K37" t="str">
+        <v>-</v>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>BR-2026-0004</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Anindita Bhattacharjee</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>1000</v>
+      </c>
+      <c r="G38" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="H38" t="str">
+        <v>anindita1603@gmail.com</v>
+      </c>
+      <c r="I38" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K38" t="str">
+        <v>-</v>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>BR-2026-0002</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Sep 30, 2026, 02:12 AM (BST)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>সাবিনা ইয়াসমিন</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>500</v>
+      </c>
+      <c r="G39" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="H39" t="str">
+        <v>sabinakakoli@gmail.com</v>
+      </c>
+      <c r="I39" t="str">
+        <v>01812345678</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K39" t="str">
+        <v>-</v>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update registration database with sent ticket records and offline attendees
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -456,13 +456,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BR-2026-0038</v>
+        <v>BR-OFFLINE-05</v>
       </c>
       <c r="C2" t="str">
-        <v>Oct 08, 2026, 08:27 PM (BST)</v>
+        <v>Oct 09, 2026, 12:26 AM (BST)</v>
       </c>
       <c r="D2" t="str">
-        <v>Tahera Jabeen</v>
+        <v>Arif Chowdhury</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -471,22 +471,22 @@
         <v>500</v>
       </c>
       <c r="G2" t="str">
-        <v>01715325576</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>taherajabeen@yahoo.com</v>
+        <v>cmarif007@gmail.com</v>
       </c>
       <c r="I2" t="str">
-        <v>01715325576</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K2" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-05</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="3">
@@ -494,31 +494,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>BR-2026-0037</v>
+        <v>BR-2026-0038</v>
       </c>
       <c r="C3" t="str">
-        <v>Oct 08, 2026, 07:42 PM (BST)</v>
+        <v>Oct 09, 2026, 12:17 AM (BST)</v>
       </c>
       <c r="D3" t="str">
-        <v>Biplob Kumar Hazra</v>
+        <v>Shanto</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G3" t="str">
-        <v>01733454575</v>
+        <v>01715008737</v>
       </c>
       <c r="H3" t="str">
-        <v>hazrabiplob@yahoo.com</v>
+        <v>kmshahriararif.shanto@gmail.com</v>
       </c>
       <c r="I3" t="str">
-        <v>01733454575</v>
+        <v>01715008737</v>
       </c>
       <c r="J3" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K3" t="str">
         <v>-</v>
@@ -532,31 +532,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>BR-2026-0036</v>
+        <v>BR-2026-0037</v>
       </c>
       <c r="C4" t="str">
-        <v>Oct 08, 2026, 05:04 PM (BST)</v>
+        <v>Oct 08, 2026, 07:42 PM (BST)</v>
       </c>
       <c r="D4" t="str">
-        <v>মাহবুবা রাখি</v>
+        <v>Biplob Kumar Hazra</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G4" t="str">
-        <v>01615253954</v>
+        <v>01733454575</v>
       </c>
       <c r="H4" t="str">
-        <v>mahbubaalam300@gmail.com</v>
+        <v>hazrabiplob@yahoo.com</v>
       </c>
       <c r="I4" t="str">
-        <v>01615253954</v>
+        <v>01733454575</v>
       </c>
       <c r="J4" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K4" t="str">
         <v>-</v>
@@ -570,7 +570,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>BR-2026-0035</v>
+        <v>BR-2026-0036</v>
       </c>
       <c r="C5" t="str">
         <v>Oct 08, 2026, 05:04 PM (BST)</v>
@@ -594,7 +594,7 @@
         <v>01615253954</v>
       </c>
       <c r="J5" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K5" t="str">
         <v>-</v>
@@ -608,10 +608,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>BR-2026-0034</v>
+        <v>BR-2026-0035</v>
       </c>
       <c r="C6" t="str">
-        <v>Oct 08, 2026, 05:03 PM (BST)</v>
+        <v>Oct 08, 2026, 05:04 PM (BST)</v>
       </c>
       <c r="D6" t="str">
         <v>মাহবুবা রাখি</v>
@@ -646,13 +646,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>BR-2026-0033</v>
+        <v>BR-2026-0034</v>
       </c>
       <c r="C7" t="str">
-        <v>Oct 08, 2026, 04:06 PM (BST)</v>
+        <v>Oct 08, 2026, 05:03 PM (BST)</v>
       </c>
       <c r="D7" t="str">
-        <v>Suraiya Mozammel</v>
+        <v>মাহবুবা রাখি</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -661,13 +661,13 @@
         <v>500</v>
       </c>
       <c r="G7" t="str">
-        <v>01712963636</v>
+        <v>01615253954</v>
       </c>
       <c r="H7" t="str">
-        <v>srabani.s@brac.net</v>
+        <v>mahbubaalam300@gmail.com</v>
       </c>
       <c r="I7" t="str">
-        <v>01717662350</v>
+        <v>01615253954</v>
       </c>
       <c r="J7" t="str">
         <v>Ticket Not Sent</v>
@@ -684,13 +684,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>BR-2026-0032</v>
+        <v>BR-2026-0033</v>
       </c>
       <c r="C8" t="str">
-        <v>Oct 08, 2026, 02:19 PM (BST)</v>
+        <v>Oct 08, 2026, 04:06 PM (BST)</v>
       </c>
       <c r="D8" t="str">
-        <v>Mohammed Shoeb</v>
+        <v>Suraiya Mozammel</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -699,13 +699,13 @@
         <v>500</v>
       </c>
       <c r="G8" t="str">
-        <v>01615253954</v>
+        <v>01712963636</v>
       </c>
       <c r="H8" t="str">
-        <v>shoeb@trtradingbd.com</v>
+        <v>srabani.s@brac.net</v>
       </c>
       <c r="I8" t="str">
-        <v>01615253954</v>
+        <v>01717662350</v>
       </c>
       <c r="J8" t="str">
         <v>Ticket Not Sent</v>
@@ -722,31 +722,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>BR-2026-0031</v>
+        <v>BR-2026-0032</v>
       </c>
       <c r="C9" t="str">
-        <v>Oct 08, 2026, 11:42 AM (BST)</v>
+        <v>Oct 08, 2026, 02:19 PM (BST)</v>
       </c>
       <c r="D9" t="str">
-        <v>Kishower Amin</v>
+        <v>Mohammed Shoeb</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G9" t="str">
-        <v>01766903903</v>
+        <v>01615253954</v>
       </c>
       <c r="H9" t="str">
-        <v>kishowerca@gmail.com</v>
+        <v>shoeb@trtradingbd.com</v>
       </c>
       <c r="I9" t="str">
-        <v>01766903903</v>
+        <v>01615253954</v>
       </c>
       <c r="J9" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K9" t="str">
         <v>-</v>
@@ -760,31 +760,31 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>BR-2026-0030</v>
+        <v>BR-2026-0031</v>
       </c>
       <c r="C10" t="str">
-        <v>Oct 07, 2026, 10:51 PM (BST)</v>
+        <v>Oct 08, 2026, 11:42 AM (BST)</v>
       </c>
       <c r="D10" t="str">
-        <v>Juthi</v>
+        <v>Kishower Amin</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G10" t="str">
-        <v>01715458432</v>
+        <v>01766903903</v>
       </c>
       <c r="H10" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>kishowerca@gmail.com</v>
       </c>
       <c r="I10" t="str">
-        <v>01715458432</v>
+        <v>01766903903</v>
       </c>
       <c r="J10" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K10" t="str">
         <v>-</v>
@@ -798,31 +798,31 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>BR-2026-0029</v>
+        <v>BR-2026-0030</v>
       </c>
       <c r="C11" t="str">
-        <v>Oct 07, 2026, 03:17 PM (BST)</v>
+        <v>Oct 07, 2026, 10:51 PM (BST)</v>
       </c>
       <c r="D11" t="str">
-        <v>Bidhan Chandra Pal</v>
+        <v>Juthi</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="G11" t="str">
-        <v>01730715222</v>
+        <v>01715458432</v>
       </c>
       <c r="H11" t="str">
-        <v>bidhan.probhaaurora@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I11" t="str">
-        <v>01730715222</v>
+        <v>01715458432</v>
       </c>
       <c r="J11" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K11" t="str">
         <v>-</v>
@@ -836,13 +836,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>BR-OFFLINE-04</v>
+        <v>BR-2026-0029</v>
       </c>
       <c r="C12" t="str">
-        <v>Oct 07, 2026, 12:01 AM (BST)</v>
+        <v>Oct 07, 2026, 03:17 PM (BST)</v>
       </c>
       <c r="D12" t="str">
-        <v>Shahajadi Begum</v>
+        <v>Bidhan Chandra Pal</v>
       </c>
       <c r="E12">
         <v>3</v>
@@ -851,22 +851,22 @@
         <v>1500</v>
       </c>
       <c r="G12" t="str">
-        <v/>
+        <v>01730715222</v>
       </c>
       <c r="H12" t="str">
-        <v>shahajadibegum@gmail.com</v>
+        <v>bidhan.probhaaurora@gmail.com</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>01730715222</v>
       </c>
       <c r="J12" t="str">
         <v>Mail Sent</v>
       </c>
       <c r="K12" t="str">
-        <v>BR-OFFLINE-04</v>
+        <v>-</v>
       </c>
       <c r="L12" t="str">
-        <v>Offline CSV registration</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -874,25 +874,25 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>BR-OFFLINE-03</v>
+        <v>BR-OFFLINE-04</v>
       </c>
       <c r="C13" t="str">
         <v>Oct 07, 2026, 12:01 AM (BST)</v>
       </c>
       <c r="D13" t="str">
-        <v>Abid Aziz</v>
+        <v>Shahajadi Begum</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F13">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G13" t="str">
         <v/>
       </c>
       <c r="H13" t="str">
-        <v>aby9029@gmail.com</v>
+        <v>shahajadibegum@gmail.com</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -901,7 +901,7 @@
         <v>Mail Sent</v>
       </c>
       <c r="K13" t="str">
-        <v>BR-OFFLINE-03</v>
+        <v>BR-OFFLINE-04</v>
       </c>
       <c r="L13" t="str">
         <v>Offline CSV registration</v>
@@ -912,37 +912,37 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>BR-2026-0026</v>
+        <v>BR-OFFLINE-03</v>
       </c>
       <c r="C14" t="str">
-        <v>Oct 06, 2026, 11:24 PM (BST)</v>
+        <v>Oct 07, 2026, 12:01 AM (BST)</v>
       </c>
       <c r="D14" t="str">
-        <v>Saud Bin Jahan (Susan)</v>
+        <v>Abid Aziz</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G14" t="str">
-        <v>01714100924</v>
+        <v/>
       </c>
       <c r="H14" t="str">
-        <v>saud.jahan@outlook.com</v>
+        <v>aby9029@gmail.com</v>
       </c>
       <c r="I14" t="str">
-        <v>01714100924</v>
+        <v/>
       </c>
       <c r="J14" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K14" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-03</v>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="15">
@@ -950,31 +950,31 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>BR-2026-0025</v>
+        <v>BR-2026-0026</v>
       </c>
       <c r="C15" t="str">
-        <v>Oct 06, 2026, 11:03 PM (BST)</v>
+        <v>Oct 06, 2026, 11:24 PM (BST)</v>
       </c>
       <c r="D15" t="str">
-        <v>Joya Tasnim</v>
+        <v>Saud Bin Jahan (Susan)</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G15" t="str">
-        <v>01911586356</v>
+        <v>01714100924</v>
       </c>
       <c r="H15" t="str">
-        <v>joyatasnim229@gmail.com</v>
+        <v>saud.jahan@outlook.com</v>
       </c>
       <c r="I15" t="str">
-        <v>01876892247</v>
+        <v>01714100924</v>
       </c>
       <c r="J15" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K15" t="str">
         <v>-</v>
@@ -988,31 +988,31 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>BR-2026-0024</v>
+        <v>BR-2026-0025</v>
       </c>
       <c r="C16" t="str">
-        <v>Oct 06, 2026, 10:23 AM (BST)</v>
+        <v>Oct 06, 2026, 11:03 PM (BST)</v>
       </c>
       <c r="D16" t="str">
-        <v>Saikat Shubhra Aich</v>
+        <v>Joya Tasnim</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G16" t="str">
-        <v>01712032080</v>
+        <v>01911586356</v>
       </c>
       <c r="H16" t="str">
-        <v>ssam99@gmail.com</v>
+        <v>joyatasnim229@gmail.com</v>
       </c>
       <c r="I16" t="str">
-        <v>01712032080</v>
+        <v>01876892247</v>
       </c>
       <c r="J16" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K16" t="str">
         <v>-</v>
@@ -1026,13 +1026,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>BR-2026-0023</v>
+        <v>BR-2026-0024</v>
       </c>
       <c r="C17" t="str">
-        <v>Oct 05, 2026, 09:13 AM (BST)</v>
+        <v>Oct 06, 2026, 10:23 AM (BST)</v>
       </c>
       <c r="D17" t="str">
-        <v>Shariful Islam</v>
+        <v>Saikat Shubhra Aich</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -1041,13 +1041,13 @@
         <v>1000</v>
       </c>
       <c r="G17" t="str">
-        <v>01778580756</v>
+        <v>01712032080</v>
       </c>
       <c r="H17" t="str">
-        <v>sharif1658@gmail.com</v>
+        <v>ssam99@gmail.com</v>
       </c>
       <c r="I17" t="str">
-        <v>01778580756</v>
+        <v>01712032080</v>
       </c>
       <c r="J17" t="str">
         <v>Ticket Not Sent</v>
@@ -1064,37 +1064,37 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>BR-2026-0022</v>
+        <v>BR-2026-0023</v>
       </c>
       <c r="C18" t="str">
-        <v>Oct 04, 2026, 05:13 PM (BST)</v>
+        <v>Oct 05, 2026, 09:13 AM (BST)</v>
       </c>
       <c r="D18" t="str">
-        <v>Mahenaw Wara</v>
+        <v>Shariful Islam</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G18" t="str">
-        <v>01030300120</v>
+        <v>01778580756</v>
       </c>
       <c r="H18" t="str">
-        <v>manana.manamaya@gmail.com</v>
+        <v>sharif1658@gmail.com</v>
       </c>
       <c r="I18" t="str">
-        <v>01030300120</v>
+        <v>01778580756</v>
       </c>
       <c r="J18" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K18" t="str">
-        <v>BR-OFFLINE-02</v>
+        <v>-</v>
       </c>
       <c r="L18" t="str">
-        <v>Offline CSV registration</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1102,13 +1102,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>BR-2026-0021</v>
+        <v>BR-2026-0022</v>
       </c>
       <c r="C19" t="str">
         <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D19" t="str">
-        <v>Ferdoushi Begum</v>
+        <v>Mahenaw Wara</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1117,19 +1117,19 @@
         <v>500</v>
       </c>
       <c r="G19" t="str">
-        <v>01717144778</v>
+        <v>01030300120</v>
       </c>
       <c r="H19" t="str">
-        <v>ferdoushi@yahoo.com</v>
+        <v>manana.manamaya@gmail.com</v>
       </c>
       <c r="I19" t="str">
-        <v>01717144778</v>
+        <v>01030300120</v>
       </c>
       <c r="J19" t="str">
         <v>Mail Sent</v>
       </c>
       <c r="K19" t="str">
-        <v>BR-OFFLINE-01</v>
+        <v>BR-OFFLINE-02</v>
       </c>
       <c r="L19" t="str">
         <v>Offline CSV registration</v>
@@ -1140,13 +1140,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>BR-2026-0020</v>
+        <v>BR-2026-0021</v>
       </c>
       <c r="C20" t="str">
-        <v>Oct 04, 2026, 11:43 AM (BST)</v>
+        <v>Oct 04, 2026, 05:13 PM (BST)</v>
       </c>
       <c r="D20" t="str">
-        <v>Delwar Hossain</v>
+        <v>Ferdoushi Begum</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1155,22 +1155,22 @@
         <v>500</v>
       </c>
       <c r="G20" t="str">
-        <v>01715458432</v>
+        <v>01717144778</v>
       </c>
       <c r="H20" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>ferdoushi@yahoo.com</v>
       </c>
       <c r="I20" t="str">
-        <v>01715458432</v>
+        <v>01717144778</v>
       </c>
       <c r="J20" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K20" t="str">
-        <v>-</v>
+        <v>BR-OFFLINE-01</v>
       </c>
       <c r="L20" t="str">
-        <v/>
+        <v>Offline CSV registration</v>
       </c>
     </row>
     <row r="21">
@@ -1178,13 +1178,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>BR-2026-0019</v>
+        <v>BR-2026-0020</v>
       </c>
       <c r="C21" t="str">
-        <v>Oct 04, 2026, 10:35 AM (BST)</v>
+        <v>Oct 04, 2026, 11:43 AM (BST)</v>
       </c>
       <c r="D21" t="str">
-        <v>ইলোরা</v>
+        <v>Delwar Hossain</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -1193,13 +1193,13 @@
         <v>500</v>
       </c>
       <c r="G21" t="str">
-        <v>01730599329</v>
+        <v>01715458432</v>
       </c>
       <c r="H21" t="str">
-        <v>sselora.harmony19@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I21" t="str">
-        <v>01730599329</v>
+        <v>01715458432</v>
       </c>
       <c r="J21" t="str">
         <v>Mail Sent</v>
@@ -1216,28 +1216,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>BR-2026-0018</v>
+        <v>BR-2026-0019</v>
       </c>
       <c r="C22" t="str">
-        <v>Oct 03, 2026, 08:34 PM (BST)</v>
+        <v>Oct 04, 2026, 10:35 AM (BST)</v>
       </c>
       <c r="D22" t="str">
-        <v>Kanika Chakraborty</v>
+        <v>ইলোরা</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G22" t="str">
-        <v>01713379897</v>
+        <v>01730599329</v>
       </c>
       <c r="H22" t="str">
-        <v>borty.kanika@yahoo.com</v>
+        <v>sselora.harmony19@gmail.com</v>
       </c>
       <c r="I22" t="str">
-        <v>01713379897</v>
+        <v>01730599329</v>
       </c>
       <c r="J22" t="str">
         <v>Mail Sent</v>
@@ -1254,28 +1254,28 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>BR-2026-0017</v>
+        <v>BR-2026-0018</v>
       </c>
       <c r="C23" t="str">
-        <v>Oct 03, 2026, 07:54 PM (BST)</v>
+        <v>Oct 03, 2026, 08:34 PM (BST)</v>
       </c>
       <c r="D23" t="str">
-        <v>Sayema Mukarrama</v>
+        <v>Kanika Chakraborty</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F23">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G23" t="str">
-        <v>01973091880</v>
+        <v>01713379897</v>
       </c>
       <c r="H23" t="str">
-        <v>sayema14bd@gmail.com</v>
+        <v>borty.kanika@yahoo.com</v>
       </c>
       <c r="I23" t="str">
-        <v>01973091880</v>
+        <v>01713379897</v>
       </c>
       <c r="J23" t="str">
         <v>Mail Sent</v>
@@ -1292,10 +1292,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>BR-2026-0016</v>
+        <v>BR-2026-0017</v>
       </c>
       <c r="C24" t="str">
-        <v>Oct 03, 2026, 07:41 PM (BST)</v>
+        <v>Oct 03, 2026, 07:54 PM (BST)</v>
       </c>
       <c r="D24" t="str">
         <v>Sayema Mukarrama</v>
@@ -1316,7 +1316,7 @@
         <v>01973091880</v>
       </c>
       <c r="J24" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K24" t="str">
         <v>-</v>
@@ -1330,13 +1330,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>BR-2026-0015</v>
+        <v>BR-2026-0016</v>
       </c>
       <c r="C25" t="str">
-        <v>Oct 03, 2026, 07:13 PM (BST)</v>
+        <v>Oct 03, 2026, 07:41 PM (BST)</v>
       </c>
       <c r="D25" t="str">
-        <v>কাজী নজরুল ইসলাম</v>
+        <v>Sayema Mukarrama</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -1345,16 +1345,16 @@
         <v>500</v>
       </c>
       <c r="G25" t="str">
-        <v>01845972555</v>
+        <v>01973091880</v>
       </c>
       <c r="H25" t="str">
-        <v>sarothy@gmail.com</v>
+        <v>sayema14bd@gmail.com</v>
       </c>
       <c r="I25" t="str">
-        <v>01845972555</v>
+        <v>01973091880</v>
       </c>
       <c r="J25" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K25" t="str">
         <v>-</v>
@@ -1368,13 +1368,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>BR-2026-0014</v>
+        <v>BR-2026-0015</v>
       </c>
       <c r="C26" t="str">
-        <v>Oct 03, 2026, 01:27 PM (BST)</v>
+        <v>Oct 03, 2026, 07:13 PM (BST)</v>
       </c>
       <c r="D26" t="str">
-        <v>444</v>
+        <v>কাজী নজরুল ইসলাম</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -1383,16 +1383,16 @@
         <v>500</v>
       </c>
       <c r="G26" t="str">
-        <v>01712345678</v>
+        <v>01845972555</v>
       </c>
       <c r="H26" t="str">
-        <v>kentkouh+otybu@gmail.com</v>
+        <v>sarothy@gmail.com</v>
       </c>
       <c r="I26" t="str">
-        <v>01712345678</v>
+        <v>01845972555</v>
       </c>
       <c r="J26" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K26" t="str">
         <v>-</v>
@@ -1406,31 +1406,31 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>BR-2026-0013</v>
+        <v>BR-2026-0014</v>
       </c>
       <c r="C27" t="str">
-        <v>Oct 03, 2026, 12:06 PM (BST)</v>
+        <v>Oct 03, 2026, 01:27 PM (BST)</v>
       </c>
       <c r="D27" t="str">
-        <v>Ferdowsi Rita</v>
+        <v>444</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G27" t="str">
-        <v>01732770345</v>
+        <v>01712345678</v>
       </c>
       <c r="H27" t="str">
-        <v>ferdowsi.rita@gmail.com</v>
+        <v>kentkouh+otybu@gmail.com</v>
       </c>
       <c r="I27" t="str">
-        <v>01732770345</v>
+        <v>01712345678</v>
       </c>
       <c r="J27" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K27" t="str">
         <v>-</v>
@@ -1444,28 +1444,28 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>BR-2026-0012</v>
+        <v>BR-2026-0013</v>
       </c>
       <c r="C28" t="str">
-        <v>Oct 02, 2026, 11:09 PM (BST)</v>
+        <v>Oct 03, 2026, 12:06 PM (BST)</v>
       </c>
       <c r="D28" t="str">
-        <v>মো: হাবিবুর রহমান শিনু</v>
+        <v>Ferdowsi Rita</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G28" t="str">
-        <v>01712286494</v>
+        <v>01732770345</v>
       </c>
       <c r="H28" t="str">
-        <v>sassybd1978@gmail.com</v>
+        <v>ferdowsi.rita@gmail.com</v>
       </c>
       <c r="I28" t="str">
-        <v>01712286494</v>
+        <v>01732770345</v>
       </c>
       <c r="J28" t="str">
         <v>Mail Sent</v>
@@ -1482,31 +1482,31 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>BR-2026-0011</v>
+        <v>BR-2026-0012</v>
       </c>
       <c r="C29" t="str">
-        <v>Oct 02, 2026, 08:09 PM (BST)</v>
+        <v>Oct 02, 2026, 11:09 PM (BST)</v>
       </c>
       <c r="D29" t="str">
-        <v>Anowar Hossain</v>
+        <v>মো: হাবিবুর রহমান শিনু</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G29" t="str">
-        <v>01711080069</v>
+        <v>01712286494</v>
       </c>
       <c r="H29" t="str">
-        <v>anowarstories@gmail.com</v>
+        <v>sassybd1978@gmail.com</v>
       </c>
       <c r="I29" t="str">
-        <v>01711080069</v>
+        <v>01712286494</v>
       </c>
       <c r="J29" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K29" t="str">
         <v>-</v>
@@ -1520,28 +1520,28 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>BR-2026-0010</v>
+        <v>BR-2026-0011</v>
       </c>
       <c r="C30" t="str">
-        <v>Oct 02, 2026, 06:31 PM (BST)</v>
+        <v>Oct 02, 2026, 08:09 PM (BST)</v>
       </c>
       <c r="D30" t="str">
-        <v>Shawli Jharna</v>
+        <v>Anowar Hossain</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G30" t="str">
-        <v>01313357635</v>
+        <v>01711080069</v>
       </c>
       <c r="H30" t="str">
-        <v>shawli.jharna@yahoo.com</v>
+        <v>anowarstories@gmail.com</v>
       </c>
       <c r="I30" t="str">
-        <v>01313357635</v>
+        <v>01711080069</v>
       </c>
       <c r="J30" t="str">
         <v>Ticket Not Sent</v>
@@ -1558,13 +1558,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>BR-2026-0009</v>
+        <v>BR-2026-0010</v>
       </c>
       <c r="C31" t="str">
-        <v>Oct 02, 2026, 04:52 PM (BST)</v>
+        <v>Oct 02, 2026, 06:31 PM (BST)</v>
       </c>
       <c r="D31" t="str">
-        <v>ফারজানা মাসুদ</v>
+        <v>Shawli Jharna</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1573,13 +1573,13 @@
         <v>500</v>
       </c>
       <c r="G31" t="str">
-        <v>01822055931</v>
+        <v>01313357635</v>
       </c>
       <c r="H31" t="str">
-        <v>farjana.masud@plpg.com.bd</v>
+        <v>shawli.jharna@yahoo.com</v>
       </c>
       <c r="I31" t="str">
-        <v>01822055931</v>
+        <v>01313357635</v>
       </c>
       <c r="J31" t="str">
         <v>Ticket Not Sent</v>
@@ -1596,13 +1596,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>BR-2026-0008</v>
+        <v>BR-2026-0009</v>
       </c>
       <c r="C32" t="str">
-        <v>Oct 02, 2026, 12:51 AM (BST)</v>
+        <v>Oct 02, 2026, 04:52 PM (BST)</v>
       </c>
       <c r="D32" t="str">
-        <v>Farhana Hafiz Tania</v>
+        <v>ফারজানা মাসুদ</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -1611,13 +1611,13 @@
         <v>500</v>
       </c>
       <c r="G32" t="str">
-        <v>01713060155</v>
+        <v>01822055931</v>
       </c>
       <c r="H32" t="str">
-        <v>fhafiz2006@gmail.com</v>
+        <v>farjana.masud@plpg.com.bd</v>
       </c>
       <c r="I32" t="str">
-        <v>01713046659</v>
+        <v>01822055931</v>
       </c>
       <c r="J32" t="str">
         <v>Ticket Not Sent</v>
@@ -1634,13 +1634,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>BR-2026-0007</v>
+        <v>BR-2026-0008</v>
       </c>
       <c r="C33" t="str">
-        <v>Oct 01, 2026, 11:38 PM (BST)</v>
+        <v>Oct 02, 2026, 12:51 AM (BST)</v>
       </c>
       <c r="D33" t="str">
-        <v>Nahida Parvin</v>
+        <v>Farhana Hafiz Tania</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -1649,16 +1649,16 @@
         <v>500</v>
       </c>
       <c r="G33" t="str">
-        <v>01764198696</v>
+        <v>01713060155</v>
       </c>
       <c r="H33" t="str">
-        <v>avra.bhattacharjee@gmail.com</v>
+        <v>fhafiz2006@gmail.com</v>
       </c>
       <c r="I33" t="str">
-        <v>01713244349</v>
+        <v>01713046659</v>
       </c>
       <c r="J33" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K33" t="str">
         <v>-</v>
@@ -1672,31 +1672,31 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>BR-2026-0006</v>
+        <v>BR-2026-0007</v>
       </c>
       <c r="C34" t="str">
-        <v>Oct 01, 2026, 05:59 PM (BST)</v>
+        <v>Oct 01, 2026, 11:38 PM (BST)</v>
       </c>
       <c r="D34" t="str">
-        <v>Moni Akter and Shela</v>
+        <v>Nahida Parvin</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G34" t="str">
-        <v>01718277527</v>
+        <v>01764198696</v>
       </c>
       <c r="H34" t="str">
-        <v>biswas.lipika05@gmail.com</v>
+        <v>avra.bhattacharjee@gmail.com</v>
       </c>
       <c r="I34" t="str">
-        <v>01715458432</v>
+        <v>01713244349</v>
       </c>
       <c r="J34" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K34" t="str">
         <v>-</v>
@@ -1710,31 +1710,31 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>BR-2026-0009</v>
+        <v>BR-2026-0006</v>
       </c>
       <c r="C35" t="str">
-        <v>Sep 30, 2026, 02:52 PM (BST)</v>
+        <v>Oct 01, 2026, 05:59 PM (BST)</v>
       </c>
       <c r="D35" t="str">
-        <v>Emon Rahman</v>
+        <v>Moni Akter and Shela</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G35" t="str">
-        <v>01971010112</v>
+        <v>01718277527</v>
       </c>
       <c r="H35" t="str">
         <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I35" t="str">
-        <v>01971010112</v>
+        <v>01715458432</v>
       </c>
       <c r="J35" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K35" t="str">
         <v>-</v>
@@ -1748,13 +1748,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>BR-2026-0008</v>
+        <v>BR-2026-0009</v>
       </c>
       <c r="C36" t="str">
-        <v>Sep 30, 2026, 01:49 PM (BST)</v>
+        <v>Sep 30, 2026, 02:52 PM (BST)</v>
       </c>
       <c r="D36" t="str">
-        <v>Ferdowsi Rita</v>
+        <v>Emon Rahman</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -1763,16 +1763,16 @@
         <v>500</v>
       </c>
       <c r="G36" t="str">
-        <v>01732770345</v>
+        <v>01971010112</v>
       </c>
       <c r="H36" t="str">
-        <v>ferdowsi.rita@gmail.com</v>
+        <v>biswas.lipika05@gmail.com</v>
       </c>
       <c r="I36" t="str">
-        <v>01732770345</v>
+        <v>01971010112</v>
       </c>
       <c r="J36" t="str">
-        <v>Ticket Not Sent</v>
+        <v>Mail Sent</v>
       </c>
       <c r="K36" t="str">
         <v>-</v>
@@ -1786,28 +1786,28 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>BR-2026-0007</v>
+        <v>BR-2026-0008</v>
       </c>
       <c r="C37" t="str">
-        <v>Sep 30, 2026, 12:03 PM (BST)</v>
+        <v>Sep 30, 2026, 01:49 PM (BST)</v>
       </c>
       <c r="D37" t="str">
-        <v>মল্লিকা</v>
+        <v>Ferdowsi Rita</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G37" t="str">
-        <v>01716550859</v>
+        <v>01732770345</v>
       </c>
       <c r="H37" t="str">
-        <v>mallikarikta142@gmail.com</v>
+        <v>ferdowsi.rita@gmail.com</v>
       </c>
       <c r="I37" t="str">
-        <v>01716550859</v>
+        <v>01732770345</v>
       </c>
       <c r="J37" t="str">
         <v>Ticket Not Sent</v>
@@ -1824,13 +1824,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>BR-2026-0004</v>
+        <v>BR-2026-0007</v>
       </c>
       <c r="C38" t="str">
-        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+        <v>Sep 30, 2026, 12:03 PM (BST)</v>
       </c>
       <c r="D38" t="str">
-        <v>Anindita Bhattacharjee</v>
+        <v>মল্লিকা</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -1839,16 +1839,16 @@
         <v>1000</v>
       </c>
       <c r="G38" t="str">
-        <v>01711107102</v>
+        <v>01716550859</v>
       </c>
       <c r="H38" t="str">
-        <v>anindita1603@gmail.com</v>
+        <v>mallikarikta142@gmail.com</v>
       </c>
       <c r="I38" t="str">
-        <v>01711107102</v>
+        <v>01716550859</v>
       </c>
       <c r="J38" t="str">
-        <v>Mail Sent</v>
+        <v>Ticket Not Sent</v>
       </c>
       <c r="K38" t="str">
         <v>-</v>
@@ -1862,42 +1862,80 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
+        <v>BR-2026-0004</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Sep 30, 2026, 09:36 AM (BST)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Anindita Bhattacharjee</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+      <c r="F39">
+        <v>1000</v>
+      </c>
+      <c r="G39" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="H39" t="str">
+        <v>anindita1603@gmail.com</v>
+      </c>
+      <c r="I39" t="str">
+        <v>01711107102</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K39" t="str">
+        <v>-</v>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
         <v>BR-2026-0002</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C40" t="str">
         <v>Sep 30, 2026, 02:12 AM (BST)</v>
       </c>
-      <c r="D39" t="str">
+      <c r="D40" t="str">
         <v>সাবিনা ইয়াসমিন</v>
       </c>
-      <c r="E39">
-        <v>1</v>
-      </c>
-      <c r="F39">
-        <v>500</v>
-      </c>
-      <c r="G39" t="str">
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>500</v>
+      </c>
+      <c r="G40" t="str">
         <v>01812345678</v>
       </c>
-      <c r="H39" t="str">
+      <c r="H40" t="str">
         <v>sabinakakoli@gmail.com</v>
       </c>
-      <c r="I39" t="str">
+      <c r="I40" t="str">
         <v>01812345678</v>
       </c>
-      <c r="J39" t="str">
-        <v>Mail Sent</v>
-      </c>
-      <c r="K39" t="str">
-        <v>-</v>
-      </c>
-      <c r="L39" t="str">
+      <c r="J40" t="str">
+        <v>Mail Sent</v>
+      </c>
+      <c r="K40" t="str">
+        <v>-</v>
+      </c>
+      <c r="L40" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>